<commit_message>
Tuan 4 + 5
</commit_message>
<xml_diff>
--- a/Phiếu_Báo Cáo Học Tập Cá Nhân Nhóm.xlsx
+++ b/Phiếu_Báo Cáo Học Tập Cá Nhân Nhóm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ANM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDBC03DF-F1C0-492B-8F6E-14B35C6CB239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388E2012-81CF-4EAF-8320-61F6BEC3B2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D15A3D2F-CAC7-4BA5-B60B-7FC4419B3D9E}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="43">
   <si>
     <t>Tuần</t>
   </si>
@@ -142,12 +142,39 @@
   <si>
     <t xml:space="preserve">2.3.4. Cách thức hoạt động và cơ chế bảo mật </t>
   </si>
+  <si>
+    <t>2.4.4.1. Thiết lập xác thực tập trung</t>
+  </si>
+  <si>
+    <t>2.4.5.1. Kịch bản 1 : Kiểm thử sự cách ly giữa VLAN Khách và VLAN Nhân Viên</t>
+  </si>
+  <si>
+    <t>2.4.4.2. Mã hóa dữ liệu truyền dẫn</t>
+  </si>
+  <si>
+    <t>2.4.5.2. Kịch bản 2 : Kiểm thử  xác thực và quyền truy cập của VLAN Nhân Viên</t>
+  </si>
+  <si>
+    <t>2.4.4.3. Kiểm soát truy cập bằng ACL</t>
+  </si>
+  <si>
+    <t>2.4.5.3. Kịch bản 3 : Bảo mật vùng Quản trị (VLAN  30)</t>
+  </si>
+  <si>
+    <t>2.4.4.4. Cách ly thiết bị (Peer-to-Peer Blocking</t>
+  </si>
+  <si>
+    <t>2.4.5.4. Kịch bản 4 : Kiểm thử hạn chế truy cập dịch vụ củ thể trên Firewall/Router</t>
+  </si>
+  <si>
+    <t>Hoàn thành chương 3 và hoàn thiện báo cáo</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +208,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -283,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -322,6 +356,42 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -331,15 +401,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -349,29 +410,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{955875A6-7E3F-464A-943B-0209AE1511DC}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -735,75 +778,75 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A2" s="28">
+      <c r="A2" s="15">
         <v>1</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="17" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="23"/>
+      <c r="D2" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="19"/>
     </row>
     <row r="3" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="17"/>
       <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="23"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="19"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29" t="s">
+      <c r="A4" s="15"/>
+      <c r="B4" s="17" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="23"/>
+      <c r="D4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="19"/>
     </row>
     <row r="5" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="19"/>
     </row>
     <row r="6" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A6" s="28"/>
-      <c r="B6" s="30" t="s">
+      <c r="A6" s="15"/>
+      <c r="B6" s="18" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="23"/>
+      <c r="D6" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A7" s="28"/>
-      <c r="B7" s="30"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="23"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="28"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="8" t="s">
         <v>8</v>
       </c>
@@ -816,31 +859,31 @@
       <c r="E8" s="7"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="28">
+      <c r="A9" s="15">
         <v>2</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="17" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="23"/>
+      <c r="D9" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="27"/>
-      <c r="E10" s="23"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="19"/>
     </row>
     <row r="11" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A11" s="28"/>
+      <c r="A11" s="15"/>
       <c r="B11" s="8" t="s">
         <v>6</v>
       </c>
@@ -853,7 +896,7 @@
       <c r="E11" s="7"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="28"/>
+      <c r="A12" s="15"/>
       <c r="B12" s="8" t="s">
         <v>7</v>
       </c>
@@ -866,7 +909,7 @@
       <c r="E12" s="7"/>
     </row>
     <row r="13" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A13" s="28"/>
+      <c r="A13" s="15"/>
       <c r="B13" s="8" t="s">
         <v>8</v>
       </c>
@@ -879,149 +922,281 @@
       <c r="E13" s="7"/>
     </row>
     <row r="14" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A14" s="14">
+      <c r="A14" s="26">
         <v>3</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="20" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="20"/>
+      <c r="D14" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="29"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="15"/>
-      <c r="B15" s="25"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="21"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="30"/>
     </row>
     <row r="16" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A16" s="15"/>
-      <c r="B16" s="26"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="22"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="31"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="15"/>
-      <c r="B17" s="24" t="s">
+      <c r="A17" s="27"/>
+      <c r="B17" s="20" t="s">
         <v>6</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="20"/>
+      <c r="D17" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="29"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="15"/>
-      <c r="B18" s="25"/>
+      <c r="A18" s="27"/>
+      <c r="B18" s="21"/>
       <c r="C18" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="18"/>
-      <c r="E18" s="21"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="30"/>
     </row>
     <row r="19" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A19" s="15"/>
-      <c r="B19" s="26"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="22"/>
       <c r="C19" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="19"/>
-      <c r="E19" s="22"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="31"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="15"/>
-      <c r="B20" s="24" t="s">
+      <c r="A20" s="27"/>
+      <c r="B20" s="20" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="20"/>
+      <c r="D20" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="29"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="15"/>
-      <c r="B21" s="25"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="21"/>
       <c r="C21" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="18"/>
-      <c r="E21" s="21"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="30"/>
     </row>
     <row r="22" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A22" s="15"/>
-      <c r="B22" s="26"/>
+      <c r="A22" s="27"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="19"/>
-      <c r="E22" s="22"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="31"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="15"/>
-      <c r="B23" s="24" t="s">
+      <c r="A23" s="27"/>
+      <c r="B23" s="20" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E23" s="20"/>
+      <c r="D23" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="29"/>
     </row>
     <row r="24" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A24" s="15"/>
-      <c r="B24" s="25"/>
+      <c r="A24" s="27"/>
+      <c r="B24" s="21"/>
       <c r="C24" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="18"/>
-      <c r="E24" s="21"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="30"/>
     </row>
     <row r="25" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
-      <c r="A25" s="16"/>
-      <c r="B25" s="26"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="22"/>
       <c r="C25" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="19"/>
-      <c r="E25" s="22"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="31"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="15">
+        <v>4</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" s="7"/>
+    </row>
+    <row r="27" spans="1:5" ht="52.2" x14ac:dyDescent="0.35">
+      <c r="A27" s="15"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="7"/>
+    </row>
+    <row r="28" spans="1:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="A28" s="15"/>
+      <c r="B28" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="7"/>
+    </row>
+    <row r="29" spans="1:5" ht="52.2" x14ac:dyDescent="0.35">
+      <c r="A29" s="15"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="7"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="15"/>
+      <c r="B30" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="7"/>
+    </row>
+    <row r="31" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
+      <c r="A31" s="15"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31" s="7"/>
+    </row>
+    <row r="32" spans="1:5" ht="34.799999999999997" x14ac:dyDescent="0.35">
+      <c r="A32" s="15"/>
+      <c r="B32" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" s="7"/>
+    </row>
+    <row r="33" spans="1:5" ht="52.2" x14ac:dyDescent="0.35">
+      <c r="A33" s="15"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" s="7"/>
+    </row>
+    <row r="34" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="15">
+        <v>5</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="7"/>
+    </row>
+    <row r="35" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="15"/>
+      <c r="B35" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="33"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="7"/>
+    </row>
+    <row r="36" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="15"/>
+      <c r="B36" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="33"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="7"/>
+    </row>
+    <row r="37" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="15"/>
+      <c r="B37" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" s="33"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="A2:A8"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="D6:D7"/>
+  <mergeCells count="35">
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="A26:A33"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B32:B33"/>
     <mergeCell ref="A14:A25"/>
     <mergeCell ref="D17:D19"/>
     <mergeCell ref="D20:D22"/>
@@ -1033,6 +1208,22 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="B23:B25"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B6:B7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>